<commit_message>
Redesign handbook as an operating system: Operating Map, role/task routing, lifecycle map
- New homepage (Operating Map) with role cards, task/event cards, S1-S8 lifecycle map, daily rhythm
- Find by role and Find by task/event routing pages (data in site_map.py)
- Grouped navigation: Start here / Run the business / Standards / Management; founder letter moved to About
- SOP control panels for SOP-A and SOP-B, SOP-A exit formula table, SOP-B case router
- Badges (Daily use, Onboarding, Internal, Customer-facing, Launch blocker, Sign-off), source-of-truth callouts, launch blockers
- Clean page URLs with redirects from old numbered URLs; link checker; Google Sheets source-of-truth template

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7M8RsDuQjwxLQxhUj3swX
</commit_message>
<xml_diff>
--- a/templates/SOP-Tracker.xlsx
+++ b/templates/SOP-Tracker.xlsx
@@ -1588,11 +1588,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="47267836"/>
-        <c:axId val="72836480"/>
+        <c:axId val="51113196"/>
+        <c:axId val="74563405"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="47267836"/>
+        <c:axId val="51113196"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1624,7 +1624,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72836480"/>
+        <c:crossAx val="74563405"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1632,7 +1632,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="72836480"/>
+        <c:axId val="74563405"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1664,7 +1664,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47267836"/>
+        <c:crossAx val="51113196"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1827,11 +1827,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="80618700"/>
-        <c:axId val="86543700"/>
+        <c:axId val="33771387"/>
+        <c:axId val="45949659"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="80618700"/>
+        <c:axId val="33771387"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1863,7 +1863,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86543700"/>
+        <c:crossAx val="45949659"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1871,7 +1871,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86543700"/>
+        <c:axId val="45949659"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1903,7 +1903,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80618700"/>
+        <c:crossAx val="33771387"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2084,11 +2084,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25406384"/>
-        <c:axId val="74536124"/>
+        <c:axId val="60274948"/>
+        <c:axId val="22215414"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25406384"/>
+        <c:axId val="60274948"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2120,7 +2120,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74536124"/>
+        <c:crossAx val="22215414"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2128,7 +2128,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="74536124"/>
+        <c:axId val="22215414"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2160,7 +2160,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25406384"/>
+        <c:crossAx val="60274948"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2341,11 +2341,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="99412785"/>
-        <c:axId val="20261757"/>
+        <c:axId val="30352715"/>
+        <c:axId val="76553423"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="99412785"/>
+        <c:axId val="30352715"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2377,7 +2377,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20261757"/>
+        <c:crossAx val="76553423"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2385,7 +2385,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20261757"/>
+        <c:axId val="76553423"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2417,7 +2417,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99412785"/>
+        <c:crossAx val="30352715"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2598,11 +2598,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="45745501"/>
-        <c:axId val="31265379"/>
+        <c:axId val="56568529"/>
+        <c:axId val="6635566"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="45745501"/>
+        <c:axId val="56568529"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2634,7 +2634,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31265379"/>
+        <c:crossAx val="6635566"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2642,7 +2642,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31265379"/>
+        <c:axId val="6635566"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2674,7 +2674,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45745501"/>
+        <c:crossAx val="56568529"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>